<commit_message>
Implemented STA Instruction. Deleted VGA Simulator
</commit_message>
<xml_diff>
--- a/Documentation/Instruction Set Design.xlsx
+++ b/Documentation/Instruction Set Design.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aivap\OneDrive\Documents\GitHub\16-Bit-TTL-CPU\Documentation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Documents\Git Repos\16-Bit-TTL-CPU\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F1ADE7F-308C-4D6D-8A59-C76DF334BE62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{287EA34E-562A-4561-B03F-81818CFB35CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{350BCA08-6DF1-4025-A66A-B8F7D0EC3F3C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{350BCA08-6DF1-4025-A66A-B8F7D0EC3F3C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="176">
   <si>
     <t>Instruction Breakdown</t>
   </si>
@@ -507,6 +507,63 @@
   </si>
   <si>
     <t>7 - 6</t>
+  </si>
+  <si>
+    <t>Bits used to select the port being interacted with.</t>
+  </si>
+  <si>
+    <t>Advanced Instructions:</t>
+  </si>
+  <si>
+    <t>Bits 15 - 12</t>
+  </si>
+  <si>
+    <t>Bits 11 - 8</t>
+  </si>
+  <si>
+    <t>OpCode</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Instruction Name</t>
+  </si>
+  <si>
+    <t>Literal Load to Accumulator</t>
+  </si>
+  <si>
+    <t>0100</t>
+  </si>
+  <si>
+    <t>Bits 7 - 4</t>
+  </si>
+  <si>
+    <t>Bits 3 - 0</t>
+  </si>
+  <si>
+    <t>0000</t>
+  </si>
+  <si>
+    <t>h'8404'</t>
+  </si>
+  <si>
+    <t>Loads a numeric value into the accumulator, as specified by the program memory</t>
+  </si>
+  <si>
+    <t>Store Accumulator in RAM</t>
+  </si>
+  <si>
+    <t>0010</t>
+  </si>
+  <si>
+    <t>0101</t>
+  </si>
+  <si>
+    <t>h'2605'</t>
+  </si>
+  <si>
+    <t>Writes the value stored in the accumulator to the location of RAM specified by the program memory</t>
   </si>
 </sst>
 </file>
@@ -535,7 +592,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -569,6 +626,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="2" tint="-0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1" tint="0.499984740745262"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -646,7 +709,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -682,6 +745,16 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1018,7 +1091,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB2EEB3E-E52D-4D62-B71D-9018D54907AF}">
-  <dimension ref="A1:Y91"/>
+  <dimension ref="A1:AH91"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.42578125" customWidth="1"/>
@@ -1027,18 +1100,23 @@
     <col min="21" max="23" width="9.140625" customWidth="1"/>
     <col min="24" max="24" width="16" customWidth="1"/>
     <col min="25" max="25" width="123.85546875" customWidth="1"/>
-    <col min="27" max="27" width="9.140625" customWidth="1"/>
-    <col min="32" max="35" width="9.140625" customWidth="1"/>
+    <col min="27" max="27" width="20" customWidth="1"/>
+    <col min="28" max="28" width="24.5703125" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="32" max="32" width="9.140625" customWidth="1"/>
+    <col min="33" max="33" width="15.85546875" customWidth="1"/>
+    <col min="34" max="34" width="83.140625" customWidth="1"/>
+    <col min="35" max="35" width="9.140625" customWidth="1"/>
     <col min="37" max="38" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:34" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="D1" s="2"/>
     </row>
-    <row r="3" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -1075,8 +1153,32 @@
       <c r="Y3" s="15" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="4" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="AA3" s="21" t="s">
+        <v>158</v>
+      </c>
+      <c r="AB3" s="22" t="s">
+        <v>163</v>
+      </c>
+      <c r="AC3" s="22" t="s">
+        <v>159</v>
+      </c>
+      <c r="AD3" s="22" t="s">
+        <v>160</v>
+      </c>
+      <c r="AE3" s="22" t="s">
+        <v>166</v>
+      </c>
+      <c r="AF3" s="22" t="s">
+        <v>167</v>
+      </c>
+      <c r="AG3" s="22" t="s">
+        <v>161</v>
+      </c>
+      <c r="AH3" s="22" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="4" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -1106,8 +1208,29 @@
       <c r="Y4" s="13" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="5" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="AB4" s="23" t="s">
+        <v>164</v>
+      </c>
+      <c r="AC4" s="20">
+        <v>1000</v>
+      </c>
+      <c r="AD4" s="20" t="s">
+        <v>165</v>
+      </c>
+      <c r="AE4" s="20" t="s">
+        <v>168</v>
+      </c>
+      <c r="AF4" s="20" t="s">
+        <v>165</v>
+      </c>
+      <c r="AG4" s="20" t="s">
+        <v>169</v>
+      </c>
+      <c r="AH4" s="23" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="5" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1134,8 +1257,29 @@
       <c r="Y5" s="14" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="6" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="AB5" s="24" t="s">
+        <v>171</v>
+      </c>
+      <c r="AC5" s="25" t="s">
+        <v>172</v>
+      </c>
+      <c r="AD5" s="25" t="s">
+        <v>172</v>
+      </c>
+      <c r="AE5" s="25" t="s">
+        <v>168</v>
+      </c>
+      <c r="AF5" s="25" t="s">
+        <v>173</v>
+      </c>
+      <c r="AG5" s="25" t="s">
+        <v>174</v>
+      </c>
+      <c r="AH5" s="24" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="6" spans="1:34" x14ac:dyDescent="0.25">
       <c r="K6" s="10"/>
       <c r="L6" s="8"/>
       <c r="M6" s="8"/>
@@ -1156,8 +1300,15 @@
       <c r="Y6" s="13" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="7" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="AB6" s="16"/>
+      <c r="AC6" s="26"/>
+      <c r="AD6" s="26"/>
+      <c r="AE6" s="26"/>
+      <c r="AF6" s="26"/>
+      <c r="AG6" s="26"/>
+      <c r="AH6" s="16"/>
+    </row>
+    <row r="7" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -1185,8 +1336,15 @@
       <c r="Y7" s="14" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="8" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="AB7" s="16"/>
+      <c r="AC7" s="26"/>
+      <c r="AD7" s="26"/>
+      <c r="AE7" s="26"/>
+      <c r="AF7" s="26"/>
+      <c r="AG7" s="26"/>
+      <c r="AH7" s="16"/>
+    </row>
+    <row r="8" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>2</v>
       </c>
@@ -1211,8 +1369,15 @@
       <c r="Y8" s="13" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="9" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="AB8" s="16"/>
+      <c r="AC8" s="26"/>
+      <c r="AD8" s="26"/>
+      <c r="AE8" s="26"/>
+      <c r="AF8" s="26"/>
+      <c r="AG8" s="26"/>
+      <c r="AH8" s="16"/>
+    </row>
+    <row r="9" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -1237,8 +1402,15 @@
       <c r="Y9" s="14" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="10" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="AB9" s="16"/>
+      <c r="AC9" s="26"/>
+      <c r="AD9" s="26"/>
+      <c r="AE9" s="26"/>
+      <c r="AF9" s="26"/>
+      <c r="AG9" s="26"/>
+      <c r="AH9" s="16"/>
+    </row>
+    <row r="10" spans="1:34" x14ac:dyDescent="0.25">
       <c r="K10" s="6"/>
       <c r="L10" s="6"/>
       <c r="M10" s="6"/>
@@ -1257,8 +1429,15 @@
       <c r="Y10" s="13" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="11" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="AB10" s="16"/>
+      <c r="AC10" s="26"/>
+      <c r="AD10" s="26"/>
+      <c r="AE10" s="26"/>
+      <c r="AF10" s="26"/>
+      <c r="AG10" s="26"/>
+      <c r="AH10" s="16"/>
+    </row>
+    <row r="11" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -1286,8 +1465,15 @@
       <c r="Y11" s="14" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="12" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="AB11" s="16"/>
+      <c r="AC11" s="26"/>
+      <c r="AD11" s="26"/>
+      <c r="AE11" s="26"/>
+      <c r="AF11" s="26"/>
+      <c r="AG11" s="26"/>
+      <c r="AH11" s="16"/>
+    </row>
+    <row r="12" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>2</v>
       </c>
@@ -1309,9 +1495,18 @@
       <c r="X12" s="13" t="s">
         <v>135</v>
       </c>
-      <c r="Y12" s="13"/>
-    </row>
-    <row r="13" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="Y12" s="13" t="s">
+        <v>157</v>
+      </c>
+      <c r="AB12" s="16"/>
+      <c r="AC12" s="26"/>
+      <c r="AD12" s="26"/>
+      <c r="AE12" s="26"/>
+      <c r="AF12" s="26"/>
+      <c r="AG12" s="26"/>
+      <c r="AH12" s="16"/>
+    </row>
+    <row r="13" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>3</v>
       </c>
@@ -1336,8 +1531,24 @@
       <c r="Y13" s="14" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="15" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="AB13" s="16"/>
+      <c r="AC13" s="26"/>
+      <c r="AD13" s="26"/>
+      <c r="AE13" s="26"/>
+      <c r="AF13" s="26"/>
+      <c r="AG13" s="26"/>
+      <c r="AH13" s="16"/>
+    </row>
+    <row r="14" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="AB14" s="16"/>
+      <c r="AC14" s="26"/>
+      <c r="AD14" s="26"/>
+      <c r="AE14" s="26"/>
+      <c r="AF14" s="26"/>
+      <c r="AG14" s="26"/>
+      <c r="AH14" s="16"/>
+    </row>
+    <row r="15" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>11</v>
       </c>
@@ -1360,8 +1571,15 @@
       <c r="Y15" s="15" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="16" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="AB15" s="16"/>
+      <c r="AC15" s="26"/>
+      <c r="AD15" s="26"/>
+      <c r="AE15" s="26"/>
+      <c r="AF15" s="26"/>
+      <c r="AG15" s="26"/>
+      <c r="AH15" s="16"/>
+    </row>
+    <row r="16" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>2</v>
       </c>
@@ -1377,8 +1595,15 @@
       <c r="Y16" s="13" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="17" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="AB16" s="16"/>
+      <c r="AC16" s="26"/>
+      <c r="AD16" s="26"/>
+      <c r="AE16" s="26"/>
+      <c r="AF16" s="26"/>
+      <c r="AG16" s="26"/>
+      <c r="AH16" s="16"/>
+    </row>
+    <row r="17" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>3</v>
       </c>
@@ -1394,8 +1619,15 @@
       <c r="Y17" s="14" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="18" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="AB17" s="16"/>
+      <c r="AC17" s="26"/>
+      <c r="AD17" s="26"/>
+      <c r="AE17" s="26"/>
+      <c r="AF17" s="26"/>
+      <c r="AG17" s="26"/>
+      <c r="AH17" s="16"/>
+    </row>
+    <row r="18" spans="1:34" x14ac:dyDescent="0.25">
       <c r="W18" s="13" t="s">
         <v>90</v>
       </c>
@@ -1405,8 +1637,15 @@
       <c r="Y18" s="13" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="19" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="AB18" s="16"/>
+      <c r="AC18" s="16"/>
+      <c r="AD18" s="16"/>
+      <c r="AE18" s="16"/>
+      <c r="AF18" s="16"/>
+      <c r="AG18" s="16"/>
+      <c r="AH18" s="16"/>
+    </row>
+    <row r="19" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>15</v>
       </c>
@@ -1425,8 +1664,15 @@
       <c r="Y19" s="14" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="20" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="AB19" s="16"/>
+      <c r="AC19" s="16"/>
+      <c r="AD19" s="16"/>
+      <c r="AE19" s="16"/>
+      <c r="AF19" s="16"/>
+      <c r="AG19" s="16"/>
+      <c r="AH19" s="16"/>
+    </row>
+    <row r="20" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>2</v>
       </c>
@@ -1443,7 +1689,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="21" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>3</v>
       </c>
@@ -1456,14 +1702,14 @@
       <c r="X21" s="14"/>
       <c r="Y21" s="14"/>
     </row>
-    <row r="22" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:34" x14ac:dyDescent="0.25">
       <c r="W22" s="13" t="s">
         <v>94</v>
       </c>
       <c r="X22" s="13"/>
       <c r="Y22" s="13"/>
     </row>
-    <row r="23" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>18</v>
       </c>
@@ -1479,7 +1725,7 @@
       <c r="X23" s="14"/>
       <c r="Y23" s="14"/>
     </row>
-    <row r="24" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>2</v>
       </c>
@@ -1488,7 +1734,7 @@
       </c>
       <c r="Y24" s="16"/>
     </row>
-    <row r="25" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>3</v>
       </c>
@@ -1497,10 +1743,10 @@
       </c>
       <c r="Y25" s="16"/>
     </row>
-    <row r="26" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:34" x14ac:dyDescent="0.25">
       <c r="Y26" s="16"/>
     </row>
-    <row r="27" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>21</v>
       </c>
@@ -1512,7 +1758,7 @@
       </c>
       <c r="Y27" s="16"/>
     </row>
-    <row r="28" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>2</v>
       </c>
@@ -1533,7 +1779,7 @@
       </c>
       <c r="Y28" s="16"/>
     </row>
-    <row r="29" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>3</v>
       </c>
@@ -1548,7 +1794,7 @@
       </c>
       <c r="Y29" s="16"/>
     </row>
-    <row r="30" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:34" x14ac:dyDescent="0.25">
       <c r="L30">
         <v>1</v>
       </c>
@@ -1559,7 +1805,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>22</v>
       </c>

</xml_diff>

<commit_message>
First Full Instruction Set
</commit_message>
<xml_diff>
--- a/Documentation/Instruction Set Design.xlsx
+++ b/Documentation/Instruction Set Design.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Documents\Git Repos\16-Bit-TTL-CPU\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{287EA34E-562A-4561-B03F-81818CFB35CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21444B29-0D2E-4B8E-AF7F-379902FBE2CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{350BCA08-6DF1-4025-A66A-B8F7D0EC3F3C}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="204">
   <si>
     <t>Instruction Breakdown</t>
   </si>
@@ -227,9 +227,6 @@
     <t>IR Clocked. Stack POP.</t>
   </si>
   <si>
-    <t>PC Stack Jump</t>
-  </si>
-  <si>
     <t>Result put in STATUS. Next Instruction.</t>
   </si>
   <si>
@@ -344,9 +341,6 @@
     <t>IR Clocked.</t>
   </si>
   <si>
-    <t>Jump Location put on</t>
-  </si>
-  <si>
     <t>Skip</t>
   </si>
   <si>
@@ -564,13 +558,103 @@
   </si>
   <si>
     <t>Writes the value stored in the accumulator to the location of RAM specified by the program memory</t>
+  </si>
+  <si>
+    <t>FFFF</t>
+  </si>
+  <si>
+    <t>100P</t>
+  </si>
+  <si>
+    <t>1ooo</t>
+  </si>
+  <si>
+    <t>Performs an arithmetic or locical operation on the accumulator with another input. Excludes the binary shift operations</t>
+  </si>
+  <si>
+    <t>II00</t>
+  </si>
+  <si>
+    <t>F indicates where data can be fetched from. Only one F should be hight at a time.</t>
+  </si>
+  <si>
+    <t>If any F is high, P and I bits should be low. If P is High, any F bits should be low.</t>
+  </si>
+  <si>
+    <t>P indicates if the input for the operation is taken from a port. Both I bits define which port the input is taken from</t>
+  </si>
+  <si>
+    <t>Complex</t>
+  </si>
+  <si>
+    <t>Arithmetic / Logic operation (Exc Shift)</t>
+  </si>
+  <si>
+    <t>Arithmetic / Logic operation with literal</t>
+  </si>
+  <si>
+    <t>1000</t>
+  </si>
+  <si>
+    <t>h'880o'</t>
+  </si>
+  <si>
+    <t>ooo Inputs determine the operation to be completed</t>
+  </si>
+  <si>
+    <t>Performs an arithmetic or locical operation on the accumulator with a literal number from program memory.</t>
+  </si>
+  <si>
+    <t>Shift Accumulator Left/Right</t>
+  </si>
+  <si>
+    <t>101r</t>
+  </si>
+  <si>
+    <t>h'080a' / h'080b'</t>
+  </si>
+  <si>
+    <t>Performs a binary shift on the accumulator. Bit r is high if a right shift is performed. Otherwise, a left shift is performed.</t>
+  </si>
+  <si>
+    <t>Move literal to port</t>
+  </si>
+  <si>
+    <t>Moves data defined in program memory to the specified port.</t>
+  </si>
+  <si>
+    <t>0P01</t>
+  </si>
+  <si>
+    <t>h'1014' / h'1054'</t>
+  </si>
+  <si>
+    <t>Only the least significant port selection bits are used, as the ports reffered to by '10' and '11' are input only.</t>
+  </si>
+  <si>
+    <t>If P is low, output to port A. If P is high, output to port B.</t>
+  </si>
+  <si>
+    <t>Call</t>
+  </si>
+  <si>
+    <t>h'8002'</t>
+  </si>
+  <si>
+    <t>Pushes the program counter to the stack, and jumps to a location defined in program memory.</t>
+  </si>
+  <si>
+    <t>Jump Location put on data bus.</t>
+  </si>
+  <si>
+    <t>PC Jump</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -587,6 +671,13 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -709,7 +800,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -757,6 +848,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1101,11 +1193,11 @@
     <col min="24" max="24" width="16" customWidth="1"/>
     <col min="25" max="25" width="123.85546875" customWidth="1"/>
     <col min="27" max="27" width="20" customWidth="1"/>
-    <col min="28" max="28" width="24.5703125" customWidth="1"/>
+    <col min="28" max="28" width="32.85546875" customWidth="1"/>
     <col min="29" max="29" width="10.28515625" customWidth="1"/>
     <col min="32" max="32" width="9.140625" customWidth="1"/>
     <col min="33" max="33" width="15.85546875" customWidth="1"/>
-    <col min="34" max="34" width="83.140625" customWidth="1"/>
+    <col min="34" max="34" width="99.28515625" customWidth="1"/>
     <col min="35" max="35" width="9.140625" customWidth="1"/>
     <col min="37" max="38" width="9.140625" customWidth="1"/>
   </cols>
@@ -1121,10 +1213,10 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C3" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="G3" t="s">
         <v>5</v>
@@ -1134,7 +1226,7 @@
       <c r="M3" s="5"/>
       <c r="N3" s="3"/>
       <c r="O3" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="P3" s="3"/>
       <c r="Q3" s="5"/>
@@ -1142,40 +1234,40 @@
       <c r="S3" s="5"/>
       <c r="U3" s="12"/>
       <c r="V3" s="12" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="W3" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="X3" s="15" t="s">
         <v>77</v>
       </c>
-      <c r="X3" s="15" t="s">
+      <c r="Y3" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="Y3" s="15" t="s">
-        <v>79</v>
-      </c>
       <c r="AA3" s="21" t="s">
+        <v>156</v>
+      </c>
+      <c r="AB3" s="22" t="s">
+        <v>161</v>
+      </c>
+      <c r="AC3" s="22" t="s">
+        <v>157</v>
+      </c>
+      <c r="AD3" s="22" t="s">
         <v>158</v>
       </c>
-      <c r="AB3" s="22" t="s">
-        <v>163</v>
-      </c>
-      <c r="AC3" s="22" t="s">
+      <c r="AE3" s="22" t="s">
+        <v>164</v>
+      </c>
+      <c r="AF3" s="22" t="s">
+        <v>165</v>
+      </c>
+      <c r="AG3" s="22" t="s">
         <v>159</v>
       </c>
-      <c r="AD3" s="22" t="s">
+      <c r="AH3" s="22" t="s">
         <v>160</v>
-      </c>
-      <c r="AE3" s="22" t="s">
-        <v>166</v>
-      </c>
-      <c r="AF3" s="22" t="s">
-        <v>167</v>
-      </c>
-      <c r="AG3" s="22" t="s">
-        <v>161</v>
-      </c>
-      <c r="AH3" s="22" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="4" spans="1:34" x14ac:dyDescent="0.25">
@@ -1183,7 +1275,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="G4" t="s">
         <v>6</v>
@@ -1193,7 +1285,7 @@
       <c r="M4" s="8"/>
       <c r="N4" s="8"/>
       <c r="O4" s="9" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="P4" s="8"/>
       <c r="Q4" s="8"/>
@@ -1203,31 +1295,31 @@
         <v>15</v>
       </c>
       <c r="X4" s="13" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="Y4" s="13" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="AB4" s="23" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="AC4" s="20">
         <v>1000</v>
       </c>
       <c r="AD4" s="20" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="AE4" s="20" t="s">
+        <v>166</v>
+      </c>
+      <c r="AF4" s="20" t="s">
+        <v>163</v>
+      </c>
+      <c r="AG4" s="20" t="s">
+        <v>167</v>
+      </c>
+      <c r="AH4" s="23" t="s">
         <v>168</v>
-      </c>
-      <c r="AF4" s="20" t="s">
-        <v>165</v>
-      </c>
-      <c r="AG4" s="20" t="s">
-        <v>169</v>
-      </c>
-      <c r="AH4" s="23" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="5" spans="1:34" x14ac:dyDescent="0.25">
@@ -1235,14 +1327,14 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="K5" s="10"/>
       <c r="L5" s="8"/>
       <c r="M5" s="8"/>
       <c r="N5" s="8"/>
       <c r="O5" s="9" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="P5" s="8"/>
       <c r="Q5" s="8"/>
@@ -1252,31 +1344,31 @@
         <v>14</v>
       </c>
       <c r="X5" s="14" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="Y5" s="14" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="AB5" s="24" t="s">
+        <v>169</v>
+      </c>
+      <c r="AC5" s="25" t="s">
+        <v>170</v>
+      </c>
+      <c r="AD5" s="25" t="s">
+        <v>170</v>
+      </c>
+      <c r="AE5" s="25" t="s">
+        <v>166</v>
+      </c>
+      <c r="AF5" s="25" t="s">
         <v>171</v>
       </c>
-      <c r="AC5" s="25" t="s">
+      <c r="AG5" s="25" t="s">
         <v>172</v>
       </c>
-      <c r="AD5" s="25" t="s">
-        <v>172</v>
-      </c>
-      <c r="AE5" s="25" t="s">
-        <v>168</v>
-      </c>
-      <c r="AF5" s="25" t="s">
+      <c r="AH5" s="24" t="s">
         <v>173</v>
-      </c>
-      <c r="AG5" s="25" t="s">
-        <v>174</v>
-      </c>
-      <c r="AH5" s="24" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="6" spans="1:34" x14ac:dyDescent="0.25">
@@ -1285,7 +1377,7 @@
       <c r="M6" s="8"/>
       <c r="N6" s="8"/>
       <c r="O6" s="9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="P6" s="8"/>
       <c r="Q6" s="8"/>
@@ -1295,18 +1387,32 @@
         <v>13</v>
       </c>
       <c r="X6" s="13" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="Y6" s="13" t="s">
-        <v>118</v>
-      </c>
-      <c r="AB6" s="16"/>
-      <c r="AC6" s="26"/>
-      <c r="AD6" s="26"/>
-      <c r="AE6" s="26"/>
-      <c r="AF6" s="26"/>
-      <c r="AG6" s="26"/>
-      <c r="AH6" s="16"/>
+        <v>116</v>
+      </c>
+      <c r="AB6" s="23" t="s">
+        <v>183</v>
+      </c>
+      <c r="AC6" s="20" t="s">
+        <v>174</v>
+      </c>
+      <c r="AD6" s="20" t="s">
+        <v>175</v>
+      </c>
+      <c r="AE6" s="20" t="s">
+        <v>178</v>
+      </c>
+      <c r="AF6" s="20" t="s">
+        <v>176</v>
+      </c>
+      <c r="AG6" s="20" t="s">
+        <v>182</v>
+      </c>
+      <c r="AH6" s="23" t="s">
+        <v>177</v>
+      </c>
     </row>
     <row r="7" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
@@ -1331,18 +1437,20 @@
         <v>12</v>
       </c>
       <c r="X7" s="14" t="s">
+        <v>95</v>
+      </c>
+      <c r="Y7" s="14" t="s">
         <v>96</v>
       </c>
-      <c r="Y7" s="14" t="s">
-        <v>97</v>
-      </c>
-      <c r="AB7" s="16"/>
-      <c r="AC7" s="26"/>
-      <c r="AD7" s="26"/>
-      <c r="AE7" s="26"/>
-      <c r="AF7" s="26"/>
-      <c r="AG7" s="26"/>
-      <c r="AH7" s="16"/>
+      <c r="AB7" s="23"/>
+      <c r="AC7" s="23"/>
+      <c r="AD7" s="23"/>
+      <c r="AE7" s="23"/>
+      <c r="AF7" s="23"/>
+      <c r="AG7" s="23"/>
+      <c r="AH7" s="23" t="s">
+        <v>179</v>
+      </c>
     </row>
     <row r="8" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
@@ -1364,18 +1472,20 @@
         <v>11</v>
       </c>
       <c r="X8" s="13" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="Y8" s="13" t="s">
-        <v>114</v>
-      </c>
-      <c r="AB8" s="16"/>
-      <c r="AC8" s="26"/>
-      <c r="AD8" s="26"/>
-      <c r="AE8" s="26"/>
-      <c r="AF8" s="26"/>
-      <c r="AG8" s="26"/>
-      <c r="AH8" s="16"/>
+        <v>112</v>
+      </c>
+      <c r="AB8" s="23"/>
+      <c r="AC8" s="23"/>
+      <c r="AD8" s="23"/>
+      <c r="AE8" s="23"/>
+      <c r="AF8" s="23"/>
+      <c r="AG8" s="23"/>
+      <c r="AH8" s="23" t="s">
+        <v>180</v>
+      </c>
     </row>
     <row r="9" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
@@ -1400,15 +1510,17 @@
         <v>16</v>
       </c>
       <c r="Y9" s="14" t="s">
-        <v>113</v>
-      </c>
-      <c r="AB9" s="16"/>
-      <c r="AC9" s="26"/>
-      <c r="AD9" s="26"/>
-      <c r="AE9" s="26"/>
-      <c r="AF9" s="26"/>
-      <c r="AG9" s="26"/>
-      <c r="AH9" s="16"/>
+        <v>111</v>
+      </c>
+      <c r="AB9" s="23"/>
+      <c r="AC9" s="23"/>
+      <c r="AD9" s="23"/>
+      <c r="AE9" s="23"/>
+      <c r="AF9" s="23"/>
+      <c r="AG9" s="23"/>
+      <c r="AH9" s="23" t="s">
+        <v>181</v>
+      </c>
     </row>
     <row r="10" spans="1:34" x14ac:dyDescent="0.25">
       <c r="K10" s="6"/>
@@ -1424,27 +1536,29 @@
         <v>9</v>
       </c>
       <c r="X10" s="13" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="Y10" s="13" t="s">
-        <v>117</v>
-      </c>
-      <c r="AB10" s="16"/>
-      <c r="AC10" s="26"/>
-      <c r="AD10" s="26"/>
-      <c r="AE10" s="26"/>
-      <c r="AF10" s="26"/>
-      <c r="AG10" s="26"/>
-      <c r="AH10" s="16"/>
+        <v>115</v>
+      </c>
+      <c r="AB10" s="23"/>
+      <c r="AC10" s="23"/>
+      <c r="AD10" s="23"/>
+      <c r="AE10" s="23"/>
+      <c r="AF10" s="23"/>
+      <c r="AG10" s="23"/>
+      <c r="AH10" s="23" t="s">
+        <v>187</v>
+      </c>
     </row>
     <row r="11" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+      <c r="A11" s="27" t="s">
         <v>8</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="27" t="s">
         <v>9</v>
       </c>
       <c r="K11" s="6"/>
@@ -1460,26 +1574,41 @@
         <v>8</v>
       </c>
       <c r="X11" s="14" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="Y11" s="14" t="s">
-        <v>155</v>
-      </c>
-      <c r="AB11" s="16"/>
-      <c r="AC11" s="26"/>
-      <c r="AD11" s="26"/>
-      <c r="AE11" s="26"/>
-      <c r="AF11" s="26"/>
-      <c r="AG11" s="26"/>
-      <c r="AH11" s="16"/>
+        <v>153</v>
+      </c>
+      <c r="AB11" s="24" t="s">
+        <v>184</v>
+      </c>
+      <c r="AC11" s="25" t="s">
+        <v>185</v>
+      </c>
+      <c r="AD11" s="25" t="s">
+        <v>185</v>
+      </c>
+      <c r="AE11" s="25" t="s">
+        <v>166</v>
+      </c>
+      <c r="AF11" s="25" t="s">
+        <v>176</v>
+      </c>
+      <c r="AG11" s="25" t="s">
+        <v>186</v>
+      </c>
+      <c r="AH11" s="24" t="s">
+        <v>188</v>
+      </c>
     </row>
     <row r="12" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+      <c r="A12" s="27" t="s">
         <v>2</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="27" t="s">
         <v>52</v>
       </c>
+      <c r="C12" s="27"/>
       <c r="K12" s="6"/>
       <c r="L12" s="6"/>
       <c r="M12" s="6"/>
@@ -1490,29 +1619,44 @@
       <c r="R12" s="6"/>
       <c r="S12" s="6"/>
       <c r="W12" s="20" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="X12" s="13" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="Y12" s="13" t="s">
-        <v>157</v>
-      </c>
-      <c r="AB12" s="16"/>
-      <c r="AC12" s="26"/>
-      <c r="AD12" s="26"/>
-      <c r="AE12" s="26"/>
-      <c r="AF12" s="26"/>
-      <c r="AG12" s="26"/>
-      <c r="AH12" s="16"/>
+        <v>155</v>
+      </c>
+      <c r="AB12" s="23" t="s">
+        <v>189</v>
+      </c>
+      <c r="AC12" s="20" t="s">
+        <v>166</v>
+      </c>
+      <c r="AD12" s="20" t="s">
+        <v>185</v>
+      </c>
+      <c r="AE12" s="20" t="s">
+        <v>166</v>
+      </c>
+      <c r="AF12" s="20" t="s">
+        <v>190</v>
+      </c>
+      <c r="AG12" s="20" t="s">
+        <v>191</v>
+      </c>
+      <c r="AH12" s="23" t="s">
+        <v>192</v>
+      </c>
     </row>
     <row r="13" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+      <c r="A13" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="27" t="s">
         <v>10</v>
       </c>
+      <c r="C13" s="27"/>
       <c r="K13" s="7"/>
       <c r="L13" s="7"/>
       <c r="M13" s="7"/>
@@ -1523,101 +1667,135 @@
       <c r="R13" s="7"/>
       <c r="S13" s="7"/>
       <c r="W13" s="19" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="X13" s="14" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="Y13" s="14" t="s">
-        <v>115</v>
-      </c>
-      <c r="AB13" s="16"/>
-      <c r="AC13" s="26"/>
-      <c r="AD13" s="26"/>
-      <c r="AE13" s="26"/>
-      <c r="AF13" s="26"/>
-      <c r="AG13" s="26"/>
-      <c r="AH13" s="16"/>
+        <v>113</v>
+      </c>
+      <c r="AB13" s="24" t="s">
+        <v>193</v>
+      </c>
+      <c r="AC13" s="25" t="s">
+        <v>185</v>
+      </c>
+      <c r="AD13" s="25" t="s">
+        <v>166</v>
+      </c>
+      <c r="AE13" s="25" t="s">
+        <v>195</v>
+      </c>
+      <c r="AF13" s="25" t="s">
+        <v>163</v>
+      </c>
+      <c r="AG13" s="25" t="s">
+        <v>196</v>
+      </c>
+      <c r="AH13" s="24" t="s">
+        <v>194</v>
+      </c>
     </row>
     <row r="14" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="AB14" s="16"/>
-      <c r="AC14" s="26"/>
-      <c r="AD14" s="26"/>
-      <c r="AE14" s="26"/>
-      <c r="AF14" s="26"/>
-      <c r="AG14" s="26"/>
-      <c r="AH14" s="16"/>
+      <c r="AB14" s="24"/>
+      <c r="AC14" s="24"/>
+      <c r="AD14" s="24"/>
+      <c r="AE14" s="24"/>
+      <c r="AF14" s="24"/>
+      <c r="AG14" s="24"/>
+      <c r="AH14" s="24" t="s">
+        <v>197</v>
+      </c>
     </row>
     <row r="15" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+      <c r="A15" s="27" t="s">
         <v>11</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="27" t="s">
         <v>13</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="27" t="s">
         <v>14</v>
       </c>
       <c r="U15" s="3"/>
       <c r="V15" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="W15" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="X15" s="15" t="s">
+        <v>77</v>
+      </c>
+      <c r="Y15" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="AB15" s="24"/>
+      <c r="AC15" s="24"/>
+      <c r="AD15" s="24"/>
+      <c r="AE15" s="24"/>
+      <c r="AF15" s="24"/>
+      <c r="AG15" s="24"/>
+      <c r="AH15" s="24" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="16" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A16" s="27" t="s">
+        <v>2</v>
+      </c>
+      <c r="B16" s="27" t="s">
+        <v>62</v>
+      </c>
+      <c r="C16" s="27"/>
+      <c r="W16" s="13" t="s">
         <v>87</v>
       </c>
-      <c r="W15" s="15" t="s">
-        <v>77</v>
-      </c>
-      <c r="X15" s="15" t="s">
-        <v>78</v>
-      </c>
-      <c r="Y15" s="15" t="s">
-        <v>79</v>
-      </c>
-      <c r="AB15" s="16"/>
-      <c r="AC15" s="26"/>
-      <c r="AD15" s="26"/>
-      <c r="AE15" s="26"/>
-      <c r="AF15" s="26"/>
-      <c r="AG15" s="26"/>
-      <c r="AH15" s="16"/>
-    </row>
-    <row r="16" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>2</v>
-      </c>
-      <c r="B16" t="s">
-        <v>62</v>
-      </c>
-      <c r="W16" s="13" t="s">
+      <c r="X16" s="13" t="s">
+        <v>101</v>
+      </c>
+      <c r="Y16" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="AB16" s="23" t="s">
+        <v>199</v>
+      </c>
+      <c r="AC16" s="20" t="s">
+        <v>185</v>
+      </c>
+      <c r="AD16" s="20" t="s">
+        <v>166</v>
+      </c>
+      <c r="AE16" s="20" t="s">
+        <v>166</v>
+      </c>
+      <c r="AF16" s="20" t="s">
+        <v>170</v>
+      </c>
+      <c r="AG16" s="20" t="s">
+        <v>200</v>
+      </c>
+      <c r="AH16" s="23" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="17" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A17" s="27" t="s">
+        <v>3</v>
+      </c>
+      <c r="B17" s="27" t="s">
+        <v>203</v>
+      </c>
+      <c r="C17" s="27"/>
+      <c r="W17" s="14" t="s">
         <v>88</v>
       </c>
-      <c r="X16" s="13" t="s">
+      <c r="X17" s="14" t="s">
         <v>103</v>
       </c>
-      <c r="Y16" s="13" t="s">
+      <c r="Y17" s="14" t="s">
         <v>104</v>
-      </c>
-      <c r="AB16" s="16"/>
-      <c r="AC16" s="26"/>
-      <c r="AD16" s="26"/>
-      <c r="AE16" s="26"/>
-      <c r="AF16" s="26"/>
-      <c r="AG16" s="26"/>
-      <c r="AH16" s="16"/>
-    </row>
-    <row r="17" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>3</v>
-      </c>
-      <c r="B17" t="s">
-        <v>63</v>
-      </c>
-      <c r="W17" s="14" t="s">
-        <v>89</v>
-      </c>
-      <c r="X17" s="14" t="s">
-        <v>105</v>
-      </c>
-      <c r="Y17" s="14" t="s">
-        <v>106</v>
       </c>
       <c r="AB17" s="16"/>
       <c r="AC17" s="26"/>
@@ -1629,13 +1807,13 @@
     </row>
     <row r="18" spans="1:34" x14ac:dyDescent="0.25">
       <c r="W18" s="13" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="X18" s="13" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="Y18" s="13" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="AB18" s="16"/>
       <c r="AC18" s="16"/>
@@ -1656,13 +1834,13 @@
         <v>17</v>
       </c>
       <c r="W19" s="14" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="X19" s="14" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="Y19" s="14" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="AB19" s="16"/>
       <c r="AC19" s="16"/>
@@ -1680,13 +1858,13 @@
         <v>51</v>
       </c>
       <c r="W20" s="13" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="X20" s="13" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="Y20" s="13" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="21" spans="1:34" x14ac:dyDescent="0.25">
@@ -1697,14 +1875,14 @@
         <v>54</v>
       </c>
       <c r="W21" s="14" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="X21" s="14"/>
       <c r="Y21" s="14"/>
     </row>
     <row r="22" spans="1:34" x14ac:dyDescent="0.25">
       <c r="W22" s="13" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="X22" s="13"/>
       <c r="Y22" s="13"/>
@@ -1720,7 +1898,7 @@
         <v>20</v>
       </c>
       <c r="W23" s="14" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="X23" s="14"/>
       <c r="Y23" s="14"/>
@@ -1747,26 +1925,26 @@
       <c r="Y26" s="16"/>
     </row>
     <row r="27" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
+      <c r="A27" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B27" s="27" t="s">
+        <v>98</v>
+      </c>
+      <c r="C27" s="27" t="s">
         <v>99</v>
       </c>
-      <c r="C27" t="s">
+      <c r="Y27" s="16"/>
+    </row>
+    <row r="28" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A28" s="27" t="s">
+        <v>2</v>
+      </c>
+      <c r="B28" s="27" t="s">
         <v>100</v>
       </c>
-      <c r="Y27" s="16"/>
-    </row>
-    <row r="28" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>2</v>
-      </c>
-      <c r="B28" t="s">
-        <v>101</v>
-      </c>
-      <c r="C28" t="s">
-        <v>102</v>
+      <c r="C28" s="27" t="s">
+        <v>202</v>
       </c>
       <c r="L28">
         <v>0</v>
@@ -1780,9 +1958,13 @@
       <c r="Y28" s="16"/>
     </row>
     <row r="29" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
+      <c r="A29" s="27" t="s">
         <v>3</v>
       </c>
+      <c r="B29" s="27" t="s">
+        <v>203</v>
+      </c>
+      <c r="C29" s="27"/>
       <c r="L29">
         <v>0</v>
       </c>
@@ -1821,15 +2003,15 @@
     </row>
     <row r="33" spans="1:18" x14ac:dyDescent="0.25">
       <c r="R33" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="34" spans="1:18" x14ac:dyDescent="0.25">
       <c r="N34" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="O34" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="R34">
         <v>1</v>
@@ -1950,13 +2132,13 @@
     </row>
     <row r="42" spans="1:18" x14ac:dyDescent="0.25">
       <c r="M42" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="N42" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="O42" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="R42">
         <v>1</v>
@@ -2036,7 +2218,7 @@
         <v>1</v>
       </c>
       <c r="R46" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
     </row>
     <row r="47" spans="1:18" x14ac:dyDescent="0.25">
@@ -2077,22 +2259,22 @@
         <v>31</v>
       </c>
       <c r="K51" t="s">
+        <v>70</v>
+      </c>
+      <c r="L51" t="s">
         <v>71</v>
       </c>
-      <c r="L51" t="s">
+      <c r="M51" t="s">
         <v>72</v>
       </c>
-      <c r="M51" t="s">
+      <c r="N51" t="s">
+        <v>75</v>
+      </c>
+      <c r="O51" t="s">
         <v>73</v>
       </c>
-      <c r="N51" t="s">
-        <v>76</v>
-      </c>
-      <c r="O51" t="s">
+      <c r="P51" t="s">
         <v>74</v>
-      </c>
-      <c r="P51" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="52" spans="1:22" x14ac:dyDescent="0.25">
@@ -2126,7 +2308,7 @@
         <v>3</v>
       </c>
       <c r="B53" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="K53">
         <v>1</v>
@@ -2332,7 +2514,7 @@
         <v>29</v>
       </c>
       <c r="S60" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="61" spans="1:22" x14ac:dyDescent="0.25">
@@ -2346,16 +2528,16 @@
         <v>29</v>
       </c>
       <c r="K61" t="s">
+        <v>70</v>
+      </c>
+      <c r="L61" t="s">
         <v>71</v>
       </c>
-      <c r="L61" t="s">
-        <v>72</v>
-      </c>
       <c r="M61" t="s">
+        <v>79</v>
+      </c>
+      <c r="N61" t="s">
         <v>80</v>
-      </c>
-      <c r="N61" t="s">
-        <v>81</v>
       </c>
       <c r="S61">
         <v>0</v>
@@ -2378,7 +2560,7 @@
         <v>0</v>
       </c>
       <c r="Q62" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="R62">
         <v>0</v>
@@ -2468,29 +2650,29 @@
         <v>1</v>
       </c>
       <c r="R65" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="67" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B67" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C67" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="68" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B68" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C68" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
     <row r="69" spans="1:18" x14ac:dyDescent="0.25">
@@ -2498,7 +2680,7 @@
         <v>2</v>
       </c>
       <c r="B69" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="70" spans="1:18" x14ac:dyDescent="0.25">
@@ -2506,29 +2688,29 @@
         <v>3</v>
       </c>
       <c r="B70" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="72" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B72" t="s">
+        <v>124</v>
+      </c>
+      <c r="C72" t="s">
         <v>126</v>
-      </c>
-      <c r="C72" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="73" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B73" t="s">
+        <v>125</v>
+      </c>
+      <c r="C73" t="s">
         <v>127</v>
-      </c>
-      <c r="C73" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="74" spans="1:18" x14ac:dyDescent="0.25">
@@ -2536,7 +2718,7 @@
         <v>2</v>
       </c>
       <c r="B74" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="75" spans="1:18" x14ac:dyDescent="0.25">
@@ -2544,18 +2726,18 @@
         <v>3</v>
       </c>
       <c r="B75" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="77" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
+        <v>128</v>
+      </c>
+      <c r="B77" t="s">
+        <v>129</v>
+      </c>
+      <c r="C77" t="s">
         <v>130</v>
-      </c>
-      <c r="B77" t="s">
-        <v>131</v>
-      </c>
-      <c r="C77" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="78" spans="1:18" x14ac:dyDescent="0.25">
@@ -2563,7 +2745,7 @@
         <v>2</v>
       </c>
       <c r="B78" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="79" spans="1:18" x14ac:dyDescent="0.25">
@@ -2571,21 +2753,21 @@
         <v>3</v>
       </c>
       <c r="B79" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="83" spans="10:14" x14ac:dyDescent="0.25">
       <c r="J83" t="s">
+        <v>147</v>
+      </c>
+      <c r="K83" t="s">
+        <v>148</v>
+      </c>
+      <c r="L83" t="s">
         <v>149</v>
       </c>
-      <c r="K83" t="s">
-        <v>150</v>
-      </c>
-      <c r="L83" t="s">
-        <v>151</v>
-      </c>
       <c r="M83" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="84" spans="10:14" x14ac:dyDescent="0.25">

</xml_diff>